<commit_message>
docs(workshop): cập nhật WS1 + WS2 cho use case đặt trước & giỏ hàng (v1.1)
REQ-08 mở rộng: khách xem cửa hàng -> mua giao tận nhà + đặt trước hàng hết.
Thêm 5 product backlog và 15 task:
- PB-33 giỏ hàng, PB-34 đặt hàng COD, PB-35 tra đơn + xác nhận đã nhận,
  PB-36 khách đặt trước (REQ-08)
- PB-37 nhân viên quản lý phiếu đặt trước + chuyển đơn (REQ-01)
Sprint 5 đổi phạm vi: bảo hành + cửa hàng online.

Tổng: 32 -> 37 backlog, 78 -> 93 task, 342 giờ. ED giữ nguyên 18/36 (hệ số 0.5)
— nhóm không đổi, chỉ thêm use case.

Đã đọc lại file xlsx sau khi sinh: VLOOKUP giãn đúng tới $L$41, TỔNG = SUM(G5:G41),
sheet 6 E2 vẫn trỏ ED!D23 (tổng điểm) chứ không phải D24 (tỷ lệ ÷36).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc-school/WORKSHOP_2_BShoes.xlsx
+++ b/doc-school/WORKSHOP_2_BShoes.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Phiên bản: v1.0 (nhánh test-api-connect)</t>
+          <t>Phiên bản: v1.1 (nhánh test-api-connect — bổ sung đặt trước &amp; giỏ hàng khách)</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1611,43 +1611,31 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>REQ-02</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Quản lý</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn quản lý sản phẩm, biến thể (màu/size), tồn kho, danh mục và thuộc tính.</t>
-        </is>
-      </c>
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-37</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Là quản lý, tôi muốn CRUD sản phẩm để quản trị danh mục hàng</t>
+          <t>Là nhân viên, tôi muốn quản lý phiếu đặt trước và chuyển thành đơn khi hàng về</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>API /san-pham-ql CRUD</t>
+          <t>API trạng thái + chuyển đơn</t>
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
@@ -1663,16 +1651,16 @@
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Màn quản lý sản phẩm</t>
+          <t>Màn quản lý đặt trước</t>
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
@@ -1688,12 +1676,12 @@
       <c r="E32" s="4" t="inlineStr"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Test CRUD sản phẩm</t>
+          <t>Test luồng đặt trước</t>
         </is>
       </c>
       <c r="H32" s="4" t="n">
@@ -1706,31 +1694,43 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>REQ-02</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Quản lý</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn quản lý sản phẩm, biến thể (màu/size), tồn kho, danh mục và thuộc tính.</t>
+        </is>
+      </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Là quản lý, tôi muốn quản lý biến thể (màu/size/giá/giá nhập)</t>
+          <t>Là quản lý, tôi muốn CRUD sản phẩm để quản trị danh mục hàng</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>API biến thể CRUD</t>
+          <t>API /san-pham-ql CRUD</t>
         </is>
       </c>
       <c r="H33" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
@@ -1746,20 +1746,20 @@
       <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Thêm cột gia_nhap</t>
+          <t>Màn quản lý sản phẩm</t>
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -1771,20 +1771,20 @@
       <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Tab Sản phẩm chi tiết</t>
+          <t>Test CRUD sản phẩm</t>
         </is>
       </c>
       <c r="H35" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>QC</t>
         </is>
       </c>
     </row>
@@ -1794,26 +1794,26 @@
       <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Là nhân viên kho, tôi muốn nhập kho để tăng tồn</t>
+          <t>Là quản lý, tôi muốn quản lý biến thể (màu/size/giá/giá nhập)</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>API POST /{id}/nhap-kho</t>
+          <t>API biến thể CRUD</t>
         </is>
       </c>
       <c r="H36" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
@@ -1829,20 +1829,20 @@
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Ô nhập kho trên form biến thể</t>
+          <t>Thêm cột gia_nhap</t>
         </is>
       </c>
       <c r="H37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -1850,32 +1850,24 @@
       <c r="A38" s="4" t="inlineStr"/>
       <c r="B38" s="4" t="inlineStr"/>
       <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>PB-13</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Là quản lý, tôi muốn quản lý danh mục và xếp sản phẩm vào danh mục</t>
-        </is>
-      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>API gán danh mục</t>
+          <t>Tab Sản phẩm chi tiết</t>
         </is>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -1883,24 +1875,32 @@
       <c r="A39" s="4" t="inlineStr"/>
       <c r="B39" s="4" t="inlineStr"/>
       <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Là nhân viên kho, tôi muốn nhập kho để tăng tồn</t>
+        </is>
+      </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Màn danh mục + gán sản phẩm</t>
+          <t>API POST /{id}/nhap-kho</t>
         </is>
       </c>
       <c r="H39" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -1908,32 +1908,24 @@
       <c r="A40" s="4" t="inlineStr"/>
       <c r="B40" s="4" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>PB-14</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Là quản lý, tôi muốn quản lý thuộc tính sản phẩm</t>
-        </is>
-      </c>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>API CRUD 8 nhóm thuộc tính</t>
+          <t>Ô nhập kho trên form biến thể</t>
         </is>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -1941,69 +1933,57 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="4" t="inlineStr"/>
       <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>PB-13</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Là quản lý, tôi muốn quản lý danh mục và xếp sản phẩm vào danh mục</t>
+        </is>
+      </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Màn thuộc tính + lọc theo loại</t>
+          <t>API gán danh mục</t>
         </is>
       </c>
       <c r="H41" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>T38</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Màn danh mục + gán sản phẩm</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>DEV2</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>REQ-03</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Nhân viên giao hàng</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn tạo và theo dõi đơn giao hàng, xử lý trả hàng và hoàn kho.</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>PB-15</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Là nhân viên, tôi muốn tạo đơn giao hàng kèm phí ship</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>T41</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>Thêm cột phi_ship + API đặt hàng</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2011,16 +1991,24 @@
       <c r="A43" s="4" t="inlineStr"/>
       <c r="B43" s="4" t="inlineStr"/>
       <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>PB-14</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Là quản lý, tôi muốn quản lý thuộc tính sản phẩm</t>
+        </is>
+      </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Tab Đặt hàng ở POS</t>
+          <t>API CRUD 8 nhóm thuộc tính</t>
         </is>
       </c>
       <c r="H43" s="4" t="n">
@@ -2028,7 +2016,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2036,57 +2024,69 @@
       <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="4" t="inlineStr"/>
       <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>PB-16</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Là nhân viên, tôi muốn cập nhật trạng thái Đã giao</t>
-        </is>
-      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>API POST /{id}/da-giao</t>
+          <t>Màn thuộc tính + lọc theo loại</t>
         </is>
       </c>
       <c r="H44" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>REQ-03</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Nhân viên giao hàng</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn tạo và theo dõi đơn giao hàng, xử lý trả hàng và hoàn kho.</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>PB-15</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Là nhân viên, tôi muốn tạo đơn giao hàng kèm phí ship</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>T41</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Thêm cột phi_ship + API đặt hàng</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
           <t>DEV1</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr"/>
-      <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>T44</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Màn theo dõi đơn giao</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2094,32 +2094,24 @@
       <c r="A46" s="4" t="inlineStr"/>
       <c r="B46" s="4" t="inlineStr"/>
       <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>PB-17</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Là quản lý, tôi muốn xử lý trả hàng và hoàn kho</t>
-        </is>
-      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>API POST /{id}/tra-hang</t>
+          <t>Tab Đặt hàng ở POS</t>
         </is>
       </c>
       <c r="H46" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2127,61 +2119,49 @@
       <c r="A47" s="4" t="inlineStr"/>
       <c r="B47" s="4" t="inlineStr"/>
       <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>PB-16</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Là nhân viên, tôi muốn cập nhật trạng thái Đã giao</t>
+        </is>
+      </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>Nút Trả hàng ở Giao hàng &amp; Lịch sử</t>
+          <t>API POST /{id}/da-giao</t>
         </is>
       </c>
       <c r="H47" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>DEV3</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>REQ-04</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Nhân viên bảo hành</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn tiếp nhận và xử lý yêu cầu bảo hành của khách.</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>PB-18</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Là NV bảo hành, tôi muốn tiếp nhận đơn bảo hành</t>
-        </is>
-      </c>
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>Bảng bao_hanh + entity/repo</t>
+          <t>Màn theo dõi đơn giao</t>
         </is>
       </c>
       <c r="H48" s="4" t="n">
@@ -2189,7 +2169,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2197,16 +2177,24 @@
       <c r="A49" s="4" t="inlineStr"/>
       <c r="B49" s="4" t="inlineStr"/>
       <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>PB-17</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Là quản lý, tôi muốn xử lý trả hàng và hoàn kho</t>
+        </is>
+      </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>API POST /api/bao-hanh</t>
+          <t>API POST /{id}/tra-hang</t>
         </is>
       </c>
       <c r="H49" s="4" t="n">
@@ -2226,49 +2214,61 @@
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Form tiếp nhận bảo hành</t>
+          <t>Nút Trả hàng ở Giao hàng &amp; Lịch sử</t>
         </is>
       </c>
       <c r="H50" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV3</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>REQ-04</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Nhân viên bảo hành</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn tiếp nhận và xử lý yêu cầu bảo hành của khách.</t>
+        </is>
+      </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-18</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Là NV bảo hành, tôi muốn cập nhật trạng thái xử lý bảo hành</t>
+          <t>Là NV bảo hành, tôi muốn tiếp nhận đơn bảo hành</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>API cập nhật trạng thái BH</t>
+          <t>Bảng bao_hanh + entity/repo</t>
         </is>
       </c>
       <c r="H51" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
@@ -2284,20 +2284,20 @@
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>Màn bảo hành master-detail</t>
+          <t>API POST /api/bao-hanh</t>
         </is>
       </c>
       <c r="H52" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2309,20 +2309,20 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>Test luồng bảo hành</t>
+          <t>Form tiếp nhận bảo hành</t>
         </is>
       </c>
       <c r="H53" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2332,22 +2332,22 @@
       <c r="C54" s="4" t="inlineStr"/>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>PB-20</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Là NV bảo hành, tôi muốn in phiếu bảo hành</t>
+          <t>Là NV bảo hành, tôi muốn cập nhật trạng thái xử lý bảo hành</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu bảo hành</t>
+          <t>API cập nhật trạng thái BH</t>
         </is>
       </c>
       <c r="H54" s="4" t="n">
@@ -2355,52 +2355,32 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>T51</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Màn bảo hành master-detail</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
           <t>DEV2</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>REQ-05</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Quản lý</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn quản lý thông tin khách hàng và địa chỉ giao hàng.</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>PB-21</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Là quản lý, tôi muốn CRUD khách hàng</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>T54</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>API khách hàng CRUD</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2412,20 +2392,20 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>Màn khách hàng</t>
+          <t>Test luồng bảo hành</t>
         </is>
       </c>
       <c r="H56" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>QC</t>
         </is>
       </c>
     </row>
@@ -2435,47 +2415,67 @@
       <c r="C57" s="4" t="inlineStr"/>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>PB-20</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Là quản lý, tôi muốn quản lý địa chỉ giao hàng của khách</t>
+          <t>Là NV bảo hành, tôi muốn in phiếu bảo hành</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>API địa chỉ CRUD</t>
+          <t>Mẫu in phiếu bảo hành</t>
         </is>
       </c>
       <c r="H57" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr"/>
-      <c r="B58" s="4" t="inlineStr"/>
-      <c r="C58" s="4" t="inlineStr"/>
-      <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="4" t="inlineStr"/>
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>REQ-05</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Quản lý</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn quản lý thông tin khách hàng và địa chỉ giao hàng.</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>PB-21</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Là quản lý, tôi muốn CRUD khách hàng</t>
+        </is>
+      </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Tab Địa chỉ trong Khách hàng</t>
+          <t>API khách hàng CRUD</t>
         </is>
       </c>
       <c r="H58" s="4" t="n">
@@ -2483,44 +2483,24 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>REQ-06</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Kế toán / Chủ shop</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn xem thống kê doanh thu, lợi nhuận, ROI để ra quyết định.</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>PB-23</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xem KPI tổng quan</t>
-        </is>
-      </c>
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Query tổng quan</t>
+          <t>Màn khách hàng</t>
         </is>
       </c>
       <c r="H59" s="4" t="n">
@@ -2528,7 +2508,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2536,24 +2516,32 @@
       <c r="A60" s="4" t="inlineStr"/>
       <c r="B60" s="4" t="inlineStr"/>
       <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="4" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>PB-22</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Là quản lý, tôi muốn quản lý địa chỉ giao hàng của khách</t>
+        </is>
+      </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Thẻ KPI trên dashboard</t>
+          <t>API địa chỉ CRUD</t>
         </is>
       </c>
       <c r="H60" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2561,57 +2549,69 @@
       <c r="A61" s="4" t="inlineStr"/>
       <c r="B61" s="4" t="inlineStr"/>
       <c r="C61" s="4" t="inlineStr"/>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>PB-24</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xem biểu đồ dòng tiền theo tháng</t>
-        </is>
-      </c>
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Query dòng tiền theo tháng</t>
+          <t>Tab Địa chỉ trong Khách hàng</t>
         </is>
       </c>
       <c r="H61" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>REQ-06</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Kế toán / Chủ shop</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn xem thống kê doanh thu, lợi nhuận, ROI để ra quyết định.</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>PB-23</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Là kế toán, tôi muốn xem KPI tổng quan</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>T58</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>Query tổng quan</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
           <t>DEV1</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr"/>
-      <c r="B62" s="4" t="inlineStr"/>
-      <c r="C62" s="4" t="inlineStr"/>
-      <c r="D62" s="4" t="inlineStr"/>
-      <c r="E62" s="4" t="inlineStr"/>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>T61</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t>Biểu đồ dòng tiền + lọc năm</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I62" s="4" t="inlineStr">
-        <is>
-          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2619,32 +2619,24 @@
       <c r="A63" s="4" t="inlineStr"/>
       <c r="B63" s="4" t="inlineStr"/>
       <c r="C63" s="4" t="inlineStr"/>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>PB-25</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xem ROI theo sản phẩm</t>
-        </is>
-      </c>
+      <c r="D63" s="4" t="inlineStr"/>
+      <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>Query ROI theo sản phẩm</t>
+          <t>Thẻ KPI trên dashboard</t>
         </is>
       </c>
       <c r="H63" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2652,24 +2644,32 @@
       <c r="A64" s="4" t="inlineStr"/>
       <c r="B64" s="4" t="inlineStr"/>
       <c r="C64" s="4" t="inlineStr"/>
-      <c r="D64" s="4" t="inlineStr"/>
-      <c r="E64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>PB-24</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Là kế toán, tôi muốn xem biểu đồ dòng tiền theo tháng</t>
+        </is>
+      </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>Biểu đồ ROI</t>
+          <t>Query dòng tiền theo tháng</t>
         </is>
       </c>
       <c r="H64" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2677,32 +2677,24 @@
       <c r="A65" s="4" t="inlineStr"/>
       <c r="B65" s="4" t="inlineStr"/>
       <c r="C65" s="4" t="inlineStr"/>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>PB-26</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xem tỷ lệ giữ chân khách hàng</t>
-        </is>
-      </c>
+      <c r="D65" s="4" t="inlineStr"/>
+      <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Query giữ chân khách</t>
+          <t>Biểu đồ dòng tiền + lọc năm</t>
         </is>
       </c>
       <c r="H65" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2710,24 +2702,32 @@
       <c r="A66" s="4" t="inlineStr"/>
       <c r="B66" s="4" t="inlineStr"/>
       <c r="C66" s="4" t="inlineStr"/>
-      <c r="D66" s="4" t="inlineStr"/>
-      <c r="E66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>PB-25</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Là kế toán, tôi muốn xem ROI theo sản phẩm</t>
+        </is>
+      </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Biểu đồ tròn giữ chân</t>
+          <t>Query ROI theo sản phẩm</t>
         </is>
       </c>
       <c r="H66" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2735,32 +2735,24 @@
       <c r="A67" s="4" t="inlineStr"/>
       <c r="B67" s="4" t="inlineStr"/>
       <c r="C67" s="4" t="inlineStr"/>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>PB-27</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xem SP bán chạy / bán chậm / xu hướng</t>
-        </is>
-      </c>
+      <c r="D67" s="4" t="inlineStr"/>
+      <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>Query bán chạy/chậm/xu hướng</t>
+          <t>Biểu đồ ROI</t>
         </is>
       </c>
       <c r="H67" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2768,16 +2760,24 @@
       <c r="A68" s="4" t="inlineStr"/>
       <c r="B68" s="4" t="inlineStr"/>
       <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr"/>
-      <c r="E68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>PB-26</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Là kế toán, tôi muốn xem tỷ lệ giữ chân khách hàng</t>
+        </is>
+      </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>3 bảng xếp hạng</t>
+          <t>Query giữ chân khách</t>
         </is>
       </c>
       <c r="H68" s="4" t="n">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>DEV2</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
@@ -2793,73 +2793,53 @@
       <c r="A69" s="4" t="inlineStr"/>
       <c r="B69" s="4" t="inlineStr"/>
       <c r="C69" s="4" t="inlineStr"/>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>PB-28</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>Là kế toán, tôi muốn xuất báo cáo ra Excel</t>
-        </is>
-      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>Xuất Excel từ dashboard</t>
+          <t>Biểu đồ tròn giữ chân</t>
         </is>
       </c>
       <c r="H69" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>DEV3</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>REQ-07</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>Quản trị viên</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn quản lý nhân viên và phân quyền truy cập theo vai trò.</t>
-        </is>
-      </c>
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr"/>
+      <c r="C70" s="4" t="inlineStr"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Là quản trị, tôi muốn CRUD nhân viên</t>
+          <t>Là kế toán, tôi muốn xem SP bán chạy / bán chậm / xu hướng</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>API nhân viên CRUD</t>
+          <t>Query bán chạy/chậm/xu hướng</t>
         </is>
       </c>
       <c r="H70" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
@@ -2875,12 +2855,12 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Màn nhân viên</t>
+          <t>3 bảng xếp hạng</t>
         </is>
       </c>
       <c r="H71" s="4" t="n">
@@ -2898,55 +2878,75 @@
       <c r="C72" s="4" t="inlineStr"/>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Là quản trị, tôi muốn phân quyền truy cập màn hình theo vai trò</t>
+          <t>Là kế toán, tôi muốn xuất báo cáo ra Excel</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Cột vai_tro.quyen + API phân quyền</t>
+          <t>Xuất Excel từ dashboard</t>
         </is>
       </c>
       <c r="H72" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>DEV3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>REQ-07</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Quản trị viên</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn quản lý nhân viên và phân quyền truy cập theo vai trò.</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>PB-29</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Là quản trị, tôi muốn CRUD nhân viên</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>T69</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>API nhân viên CRUD</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I72" s="4" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>DEV1</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr"/>
-      <c r="B73" s="4" t="inlineStr"/>
-      <c r="C73" s="4" t="inlineStr"/>
-      <c r="D73" s="4" t="inlineStr"/>
-      <c r="E73" s="4" t="inlineStr"/>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>T72</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>Màn phân quyền</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2958,12 +2958,12 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Ẩn menu &amp; chặn route theo quyền</t>
+          <t>Màn nhân viên</t>
         </is>
       </c>
       <c r="H74" s="4" t="n">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>DEV3</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -2979,69 +2979,57 @@
       <c r="A75" s="4" t="inlineStr"/>
       <c r="B75" s="4" t="inlineStr"/>
       <c r="C75" s="4" t="inlineStr"/>
-      <c r="D75" s="4" t="inlineStr"/>
-      <c r="E75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>PB-30</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Là quản trị, tôi muốn phân quyền truy cập màn hình theo vai trò</t>
+        </is>
+      </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Test phân quyền</t>
+          <t>Cột vai_tro.quyen + API phân quyền</t>
         </is>
       </c>
       <c r="H75" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>DEV1</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>REQ-08</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>Khách hàng</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Tôi muốn xem cửa hàng online để chọn giày trước khi tới mua.</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>PB-31</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>Là khách hàng, tôi muốn xem trang chủ cửa hàng</t>
-        </is>
-      </c>
+      <c r="A76" s="4" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr"/>
+      <c r="C76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr"/>
+      <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>API sản phẩm cho trang chủ</t>
+          <t>Màn phân quyền</t>
         </is>
       </c>
       <c r="H76" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>DEV2</t>
         </is>
       </c>
     </row>
@@ -3053,88 +3041,515 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
+          <t>T73</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>Ẩn menu &amp; chặn route theo quyền</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>DEV3</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr"/>
+      <c r="B78" s="4" t="inlineStr"/>
+      <c r="C78" s="4" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr"/>
+      <c r="E78" s="4" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>T74</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Test phân quyền</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Tôi muốn xem cửa hàng online, đặt mua giao tận nhà và đặt trước mẫu đang hết hàng.</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>PB-31</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn xem trang chủ cửa hàng</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>T75</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>API sản phẩm cho trang chủ</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr"/>
+      <c r="B80" s="4" t="inlineStr"/>
+      <c r="C80" s="4" t="inlineStr"/>
+      <c r="D80" s="4" t="inlineStr"/>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
           <t>T76</t>
         </is>
       </c>
-      <c r="G77" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>Trang chủ cửa hàng</t>
         </is>
       </c>
-      <c r="H77" s="4" t="n">
+      <c r="H80" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I77" s="4" t="inlineStr">
+      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>DEV2</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr"/>
+      <c r="C81" s="4" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn thêm giày vào giỏ hàng</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>T79</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>API /san-pham-chi-tiet/store</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr"/>
+      <c r="B82" s="4" t="inlineStr"/>
+      <c r="C82" s="4" t="inlineStr"/>
+      <c r="D82" s="4" t="inlineStr"/>
+      <c r="E82" s="4" t="inlineStr"/>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>T80</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Composable useCart</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr"/>
+      <c r="B83" s="4" t="inlineStr"/>
+      <c r="C83" s="4" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr"/>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>T81</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Nút Thêm vào giỏ ở trang chủ</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr"/>
+      <c r="B84" s="4" t="inlineStr"/>
+      <c r="C84" s="4" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt hàng giao tận nhà (COD)</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>T82</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>API POST /gio-hang/checkout</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr"/>
+      <c r="B85" s="4" t="inlineStr"/>
+      <c r="C85" s="4" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr"/>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>T83</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Màn giỏ hàng + form nhận hàng</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr"/>
+      <c r="B86" s="4" t="inlineStr"/>
+      <c r="C86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr"/>
+      <c r="E86" s="4" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>T84</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>Test đặt hàng online</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr"/>
+      <c r="B87" s="4" t="inlineStr"/>
+      <c r="C87" s="4" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn tra cứu đơn của tôi và xác nhận đã nhận</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>T85</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>API GET /gio-hang/don-hang</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr"/>
+      <c r="B88" s="4" t="inlineStr"/>
+      <c r="C88" s="4" t="inlineStr"/>
+      <c r="D88" s="4" t="inlineStr"/>
+      <c r="E88" s="4" t="inlineStr"/>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>T86</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>API PUT /gio-hang/nhan-hang/{id}</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr"/>
+      <c r="B89" s="4" t="inlineStr"/>
+      <c r="C89" s="4" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr"/>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>T87</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>Tab Đơn của tôi</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr"/>
+      <c r="B90" s="4" t="inlineStr"/>
+      <c r="C90" s="4" t="inlineStr"/>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt trước mẫu đang hết hàng</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>T88</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>Bảng dat_truoc + entity/repo</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr"/>
+      <c r="B91" s="4" t="inlineStr"/>
+      <c r="C91" s="4" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr"/>
+      <c r="E91" s="4" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>T89</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>API POST /api/dat-truoc</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr"/>
+      <c r="B92" s="4" t="inlineStr"/>
+      <c r="C92" s="4" t="inlineStr"/>
+      <c r="D92" s="4" t="inlineStr"/>
+      <c r="E92" s="4" t="inlineStr"/>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>T90</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>Nút + modal Đặt trước ở trang chủ</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>REQ-09</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>Quản lý</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Tôi muốn quản lý phiếu giảm giá / khuyến mãi.</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D93" s="4" t="inlineStr">
         <is>
           <t>PB-32</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="E93" s="4" t="inlineStr">
         <is>
           <t>Là quản lý, tôi muốn quản lý phiếu giảm giá</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="F93" s="4" t="inlineStr">
         <is>
           <t>T77</t>
         </is>
       </c>
-      <c r="G78" s="4" t="inlineStr">
+      <c r="G93" s="4" t="inlineStr">
         <is>
           <t>API phiếu giảm giá CRUD</t>
         </is>
       </c>
-      <c r="H78" s="4" t="n">
+      <c r="H93" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I78" s="4" t="inlineStr">
+      <c r="I93" s="4" t="inlineStr">
         <is>
           <t>DEV1</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr"/>
-      <c r="B79" s="4" t="inlineStr"/>
-      <c r="C79" s="4" t="inlineStr"/>
-      <c r="D79" s="4" t="inlineStr"/>
-      <c r="E79" s="4" t="inlineStr"/>
-      <c r="F79" s="4" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr"/>
+      <c r="B94" s="4" t="inlineStr"/>
+      <c r="C94" s="4" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr"/>
+      <c r="E94" s="4" t="inlineStr"/>
+      <c r="F94" s="4" t="inlineStr">
         <is>
           <t>T78</t>
         </is>
       </c>
-      <c r="G79" s="4" t="inlineStr">
+      <c r="G94" s="4" t="inlineStr">
         <is>
           <t>Màn khuyến mãi</t>
         </is>
       </c>
-      <c r="H79" s="4" t="n">
+      <c r="H94" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I79" s="4" t="inlineStr">
+      <c r="I94" s="4" t="inlineStr">
         <is>
           <t>DEV2</t>
         </is>
@@ -3151,7 +3566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3241,7 +3656,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="5">
-        <f>VLOOKUP(B2,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B2,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3280,7 +3695,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="5">
-        <f>VLOOKUP(B3,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B3,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3319,7 +3734,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="5">
-        <f>VLOOKUP(B4,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B4,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3358,7 +3773,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="5">
-        <f>VLOOKUP(B5,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B5,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3397,7 +3812,7 @@
         <v>3</v>
       </c>
       <c r="H6" s="5">
-        <f>VLOOKUP(B6,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B6,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3436,7 +3851,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="5">
-        <f>VLOOKUP(B7,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B7,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3475,7 +3890,7 @@
         <v>3</v>
       </c>
       <c r="H8" s="5">
-        <f>VLOOKUP(B8,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B8,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3514,7 +3929,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="5">
-        <f>VLOOKUP(B9,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B9,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3553,7 +3968,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="5">
-        <f>VLOOKUP(B10,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B10,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3592,7 +4007,7 @@
         <v>2</v>
       </c>
       <c r="H11" s="5">
-        <f>VLOOKUP(B11,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B11,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3631,7 +4046,7 @@
         <v>2</v>
       </c>
       <c r="H12" s="5">
-        <f>VLOOKUP(B12,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B12,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3670,7 +4085,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="5">
-        <f>VLOOKUP(B13,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B13,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3709,7 +4124,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="5">
-        <f>VLOOKUP(B14,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B14,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3748,7 +4163,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="5">
-        <f>VLOOKUP(B15,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B15,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3787,7 +4202,7 @@
         <v>4</v>
       </c>
       <c r="H16" s="5">
-        <f>VLOOKUP(B16,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B16,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3826,7 +4241,7 @@
         <v>4</v>
       </c>
       <c r="H17" s="5">
-        <f>VLOOKUP(B17,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B17,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3865,7 +4280,7 @@
         <v>4</v>
       </c>
       <c r="H18" s="5">
-        <f>VLOOKUP(B18,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B18,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3904,7 +4319,7 @@
         <v>5</v>
       </c>
       <c r="H19" s="5">
-        <f>VLOOKUP(B19,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B19,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3943,7 +4358,7 @@
         <v>5</v>
       </c>
       <c r="H20" s="5">
-        <f>VLOOKUP(B20,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B20,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -3982,7 +4397,7 @@
         <v>5</v>
       </c>
       <c r="H21" s="5">
-        <f>VLOOKUP(B21,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B21,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4021,7 +4436,7 @@
         <v>4</v>
       </c>
       <c r="H22" s="5">
-        <f>VLOOKUP(B22,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B22,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4060,7 +4475,7 @@
         <v>4</v>
       </c>
       <c r="H23" s="5">
-        <f>VLOOKUP(B23,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B23,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4099,7 +4514,7 @@
         <v>6</v>
       </c>
       <c r="H24" s="5">
-        <f>VLOOKUP(B24,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B24,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4138,7 +4553,7 @@
         <v>6</v>
       </c>
       <c r="H25" s="5">
-        <f>VLOOKUP(B25,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B25,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4177,7 +4592,7 @@
         <v>6</v>
       </c>
       <c r="H26" s="5">
-        <f>VLOOKUP(B26,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B26,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4216,7 +4631,7 @@
         <v>6</v>
       </c>
       <c r="H27" s="5">
-        <f>VLOOKUP(B27,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B27,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4255,7 +4670,7 @@
         <v>6</v>
       </c>
       <c r="H28" s="5">
-        <f>VLOOKUP(B28,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B28,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4294,7 +4709,7 @@
         <v>6</v>
       </c>
       <c r="H29" s="5">
-        <f>VLOOKUP(B29,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B29,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4333,7 +4748,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="5">
-        <f>VLOOKUP(B30,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B30,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4372,7 +4787,7 @@
         <v>1</v>
       </c>
       <c r="H31" s="5">
-        <f>VLOOKUP(B31,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B31,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4411,7 +4826,7 @@
         <v>5</v>
       </c>
       <c r="H32" s="5">
-        <f>VLOOKUP(B32,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B32,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4450,18 +4865,213 @@
         <v>4</v>
       </c>
       <c r="H33" s="5">
-        <f>VLOOKUP(B33,'6. Ước lượng Story'!$A$5:$L$36,12,FALSE)</f>
+        <f>VLOOKUP(B33,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="G34" s="2" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>KH</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn thêm giày vào giỏ hàng</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Giỏ lưu ở trình duyệt, sửa số lượng, chặn vượt tồn kho</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" s="5">
+        <f>VLOOKUP(B34,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>KH</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt hàng giao tận nhà (COD)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Nhập người nhận/SĐT/địa chỉ, tạo đơn Chờ giao, trừ kho</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H35" s="5">
+        <f>VLOOKUP(B35,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>KH</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn tra cứu đơn của tôi và xác nhận đã nhận</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Tra theo SĐT, xem trạng thái, bấm Đã nhận hàng</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H36" s="5">
+        <f>VLOOKUP(B36,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>KH</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt trước mẫu đang hết hàng</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ cho đặt khi tồn = 0, để lại SĐT, xem số người đang chờ</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H37" s="5">
+        <f>VLOOKUP(B37,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>REQ-01</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>PB-37</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Là nhân viên, tôi muốn quản lý phiếu đặt trước và chuyển thành đơn khi hàng về</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Tab trạng thái, báo khách có hàng, chuyển phiếu thành hóa đơn giữ hàng</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H38" s="5">
+        <f>VLOOKUP(B38,'6. Ước lượng Story'!$A$5:$L$41,12,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="H34" s="2">
-        <f>SUM(H2:H33)</f>
+      <c r="H39" s="2">
+        <f>SUM(H2:H38)</f>
         <v/>
       </c>
     </row>
@@ -4532,15 +5142,15 @@
         </is>
       </c>
       <c r="C4" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,1)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,1)</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,1,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,1,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,1,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,1,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4556,15 +5166,15 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,2)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,2)</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,2,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,2,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,2,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,2,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4580,15 +5190,15 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,3)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,3)</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,3,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,3,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,3,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,3,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4604,15 +5214,15 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,4)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,4)</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,4,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,4,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,4,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,4,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4624,19 +5234,19 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Bảo hành &amp; trang chủ cửa hàng</t>
+          <t>Bảo hành &amp; cửa hàng online: trang chủ, giỏ hàng, đặt hàng COD, đặt trước</t>
         </is>
       </c>
       <c r="C8" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,5)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,5)</f>
         <v/>
       </c>
       <c r="D8" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,5,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,5,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E8" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,5,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,5,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4652,15 +5262,15 @@
         </is>
       </c>
       <c r="C9" s="4">
-        <f>COUNTIF('2. Product Backlog'!$G$2:$G$33,6)</f>
+        <f>COUNTIF('2. Product Backlog'!$G$2:$G$38,6)</f>
         <v/>
       </c>
       <c r="D9" s="4">
-        <f>SUMIF('2. Product Backlog'!$G$2:$G$33,6,'2. Product Backlog'!$H$2:$H$33)</f>
+        <f>SUMIF('2. Product Backlog'!$G$2:$G$38,6,'2. Product Backlog'!$H$2:$H$38)</f>
         <v/>
       </c>
       <c r="E9" s="4">
-        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$79,6,'4. Sprint Backlog'!$E$2:$E$79)</f>
+        <f>SUMIF('4. Sprint Backlog'!$G$2:$G$94,6,'4. Sprint Backlog'!$E$2:$E$94)</f>
         <v/>
       </c>
     </row>
@@ -4694,7 +5304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7714,13 +8324,583 @@
       </c>
     </row>
     <row r="80">
-      <c r="D80" s="2" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>T79</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>API /san-pham-chi-tiet/store</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Catalogue giữ cả SP hết hàng cho trang chủ</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>T80</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Composable useCart</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Giỏ ở localStorage, cộng/trừ/xóa, chặn vượt tồn</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>T81</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Nút Thêm vào giỏ ở trang chủ</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Gắn giỏ thật, badge số lượng trên header</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>T82</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>API POST /gio-hang/checkout</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Tạo đơn Chờ giao, COD, trừ kho nguyên tử từng dòng</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>T83</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Màn giỏ hàng + form nhận hàng</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Bảng dòng hàng, sửa SL, form tên/SĐT/địa chỉ</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>T84</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Test đặt hàng online</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Đủ hàng / thiếu hàng / thiếu thông tin</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>T85</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>API GET /gio-hang/don-hang</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Tra đơn theo SĐT, bỏ hóa đơn nháp tại quầy</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>T86</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>API PUT /gio-hang/nhan-hang/{id}</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Dùng lại daGiao: Chờ giao -&gt; Đã giao + lịch sử</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>T87</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Tab Đơn của tôi</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Tra theo SĐT, danh sách + nút Đã nhận hàng</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>T88</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Bảng dat_truoc + entity/repo</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>CSDL mới cho đặt trước</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>T89</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>API POST /api/dat-truoc</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ cho đăng ký khi tồn = 0, sinh mã phiếu</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>T90</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Nút + modal Đặt trước ở trang chủ</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>SP hết hàng: ảnh xám, form đăng ký, số người chờ</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>T91</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>PB-37</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>API trạng thái + chuyển đơn</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>PUT trạng thái, POST chuyển phiếu thành hóa đơn giữ hàng</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>DEV1</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>T92</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>PB-37</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Màn quản lý đặt trước</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>4 tab trạng thái + panel chi tiết + chuyển đơn</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>DEV2</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>T93</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>PB-37</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Test luồng đặt trước</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Đặt -&gt; có hàng -&gt; chuyển đơn -&gt; trừ kho</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>TỔNG GIỜ</t>
         </is>
       </c>
-      <c r="E80" s="2">
-        <f>SUM(E2:E79)</f>
+      <c r="E95" s="2">
+        <f>SUM(E2:E94)</f>
         <v/>
       </c>
     </row>
@@ -8377,7 +9557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10029,21 +11209,261 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="2" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>PB-33</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn thêm giày vào giỏ hàng</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="5">
+        <f>SUM(C37:F37)</f>
+        <v/>
+      </c>
+      <c r="H37" s="5">
+        <f>$C$2</f>
+        <v/>
+      </c>
+      <c r="I37" s="5">
+        <f>G37*H37</f>
+        <v/>
+      </c>
+      <c r="J37" s="5">
+        <f>$E$2</f>
+        <v/>
+      </c>
+      <c r="K37" s="11">
+        <f>I37*J37/36</f>
+        <v/>
+      </c>
+      <c r="L37" s="5">
+        <f>IF(K37&lt;=1,1,IF(K37&lt;=2,2,IF(K37&lt;=3,3,IF(K37&lt;=5,5,IF(K37&lt;=8,8,IF(K37&lt;=13,13,21))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>PB-34</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt hàng giao tận nhà (COD)</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="5">
+        <f>SUM(C38:F38)</f>
+        <v/>
+      </c>
+      <c r="H38" s="5">
+        <f>$C$2</f>
+        <v/>
+      </c>
+      <c r="I38" s="5">
+        <f>G38*H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="5">
+        <f>$E$2</f>
+        <v/>
+      </c>
+      <c r="K38" s="11">
+        <f>I38*J38/36</f>
+        <v/>
+      </c>
+      <c r="L38" s="5">
+        <f>IF(K38&lt;=1,1,IF(K38&lt;=2,2,IF(K38&lt;=3,3,IF(K38&lt;=5,5,IF(K38&lt;=8,8,IF(K38&lt;=13,13,21))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>PB-35</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn tra cứu đơn của tôi và xác nhận đã nhận</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="5">
+        <f>SUM(C39:F39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="5">
+        <f>$C$2</f>
+        <v/>
+      </c>
+      <c r="I39" s="5">
+        <f>G39*H39</f>
+        <v/>
+      </c>
+      <c r="J39" s="5">
+        <f>$E$2</f>
+        <v/>
+      </c>
+      <c r="K39" s="11">
+        <f>I39*J39/36</f>
+        <v/>
+      </c>
+      <c r="L39" s="5">
+        <f>IF(K39&lt;=1,1,IF(K39&lt;=2,2,IF(K39&lt;=3,3,IF(K39&lt;=5,5,IF(K39&lt;=8,8,IF(K39&lt;=13,13,21))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Là khách hàng, tôi muốn đặt trước mẫu đang hết hàng</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="5">
+        <f>SUM(C40:F40)</f>
+        <v/>
+      </c>
+      <c r="H40" s="5">
+        <f>$C$2</f>
+        <v/>
+      </c>
+      <c r="I40" s="5">
+        <f>G40*H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="5">
+        <f>$E$2</f>
+        <v/>
+      </c>
+      <c r="K40" s="11">
+        <f>I40*J40/36</f>
+        <v/>
+      </c>
+      <c r="L40" s="5">
+        <f>IF(K40&lt;=1,1,IF(K40&lt;=2,2,IF(K40&lt;=3,3,IF(K40&lt;=5,5,IF(K40&lt;=8,8,IF(K40&lt;=13,13,21))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>PB-37</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Là nhân viên, tôi muốn quản lý phiếu đặt trước và chuyển thành đơn khi hàng về</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="5">
+        <f>SUM(C41:F41)</f>
+        <v/>
+      </c>
+      <c r="H41" s="5">
+        <f>$C$2</f>
+        <v/>
+      </c>
+      <c r="I41" s="5">
+        <f>G41*H41</f>
+        <v/>
+      </c>
+      <c r="J41" s="5">
+        <f>$E$2</f>
+        <v/>
+      </c>
+      <c r="K41" s="11">
+        <f>I41*J41/36</f>
+        <v/>
+      </c>
+      <c r="L41" s="5">
+        <f>IF(K41&lt;=1,1,IF(K41&lt;=2,2,IF(K41&lt;=3,3,IF(K41&lt;=5,5,IF(K41&lt;=8,8,IF(K41&lt;=13,13,21))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="G37" s="2">
-        <f>SUM(G5:G36)</f>
-        <v/>
-      </c>
-      <c r="K37" s="12">
-        <f>SUM(K5:K36)</f>
-        <v/>
-      </c>
-      <c r="L37" s="2">
-        <f>SUM(L5:L36)</f>
+      <c r="G42" s="2">
+        <f>SUM(G5:G41)</f>
+        <v/>
+      </c>
+      <c r="K42" s="12">
+        <f>SUM(K5:K41)</f>
+        <v/>
+      </c>
+      <c r="L42" s="2">
+        <f>SUM(L5:L41)</f>
         <v/>
       </c>
     </row>

</xml_diff>